<commit_message>
Ajout des fichiers test cases
</commit_message>
<xml_diff>
--- a/test-cases/test-cases.xlsx
+++ b/test-cases/test-cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projets\Miniprojet-QA\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB7E8FB-55D6-448F-BD6B-BAD4A054AFC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9072B942-B82E-4ECC-84C8-82730A8341F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{13BA0E36-25A6-45AD-A3DF-7CF1EDF8E77E}"/>
   </bookViews>
@@ -788,7 +788,7 @@
       <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F2" s="4" t="s">

</xml_diff>